<commit_message>
doc: translate cell B1 of Example sheet to English in Lieferantenabfrage_Template_en.xlsx
</commit_message>
<xml_diff>
--- a/Meilenstein 1/Lieferantenabfrage_Template_en.xlsx
+++ b/Meilenstein 1/Lieferantenabfrage_Template_en.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ausfüllbeispiel für einen Musterartikel</t>
+          <t>Example Entry for a Sample Product</t>
         </is>
       </c>
       <c r="C1" s="7" t="inlineStr">
@@ -740,13 +740,13 @@
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Brand" prompt="Please enter the short brand name to be shown on the label (e.g. &quot;Miele&quot; instead of &quot;Miele GmbH&quot;)."/>
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Model Identifier" prompt="Please enter the exact manufacturer model code (e.g. &quot;WXD160&quot;)."/>
-    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Value" error="Please enter a whole number greater than 2 (e.g. 3, 5, 10)." promptTitle="Manufacturer Warranty" prompt="Please enter the warranty period in years as a whole number only (e.g., 3, 5, 10). Do not write &quot;years&quot; or &quot;y&quot;." type="whole" operator="greaterThan">
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" promptTitle="Brand" prompt="Please enter the short brand name to be shown on the label (e.g. &quot;Miele&quot; instead of &quot;Miele GmbH&quot;)."/>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" promptTitle="Model Identifier" prompt="Please enter the exact manufacturer model code (e.g. &quot;WXD160&quot;)."/>
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Value" error="Please enter a whole number greater than 2 (e.g. 3, 5, 10)." promptTitle="Manufacturer Warranty" prompt="Please enter the warranty period in years as a whole number only (e.g., 3, 5, 10). Do not write &quot;years&quot; or &quot;y&quot;." type="whole" operator="greaterThan">
       <formula1>2</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Link to Warranty Conditions" prompt="Please enter the direct URL link to the warranty conditions on your website (e.g., https://www.manufacturer.com/warranty). Do not write free text like &quot;in the box&quot;."/>
-    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Selection" error="Invalid selection. Please select Yes or No from the dropdown menu." promptTitle="Warranty Confirmation" prompt="Please select &quot;Yes&quot; or &quot;No&quot; from the dropdown menu." type="list">
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" promptTitle="Link to Warranty Conditions" prompt="Please enter the direct URL link to the warranty conditions on your website (e.g., https://www.manufacturer.com/warranty). Do not write free text like &quot;in the box&quot;."/>
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Selection" error="Invalid selection. Please select Yes or No from the dropdown menu." promptTitle="Warranty Confirmation" prompt="Please select &quot;Yes&quot; or &quot;No&quot; from the dropdown menu." type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>